<commit_message>
update: sync latest RELP_Configuration.xlsx from RELP_3
</commit_message>
<xml_diff>
--- a/RELP_Configuration.xlsx
+++ b/RELP_Configuration.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView windowHeight="15380" activeTab="9"/>
+    <workbookView windowHeight="15380" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Auto Run" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1522" uniqueCount="443">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1523" uniqueCount="444">
   <si>
     <t>Factory</t>
   </si>
@@ -1065,7 +1065,10 @@
     <t xml:space="preserve">[max_weight =100, decay_rate =0.75, reverse = True, defect_pct = True, multiplier =1] </t>
   </si>
   <si>
-    <t xml:space="preserve">[max_weight =100, decay_rate =1.5, reverse = True, multiplier =1] </t>
+    <t>[0.01, 0.02, 0.03, 0.04, 0.05, 0.06, 0.07, 0.08, 0.09, 0.10, 0.11, 0.13, 0.15, 0.17, 0.19, 0.21, 0.23, 0.25, 0.27, 0.29, 0.31]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[max_weight =100, decay_rate =0.3, reverse = True, defect_pct = True, multiplier =1] </t>
   </si>
   <si>
     <t>Block Size</t>
@@ -1384,7 +1387,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="25">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1395,13 +1398,6 @@
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -1894,28 +1890,31 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="44" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="177" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="42" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1924,118 +1923,115 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -2048,17 +2044,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2557,19 +2553,19 @@
         <v>8</v>
       </c>
       <c r="D1" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E1" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="F1" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G1" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="H1" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -2720,7 +2716,7 @@
         <v>2026</v>
       </c>
       <c r="C12" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="E12">
         <v>0.01</v>
@@ -2734,7 +2730,7 @@
         <v>2026</v>
       </c>
       <c r="C13" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="E13">
         <v>0.01</v>
@@ -2762,7 +2758,7 @@
         <v>2026</v>
       </c>
       <c r="C15" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="E15">
         <v>0.05</v>
@@ -2829,19 +2825,19 @@
         <v>8</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -2855,13 +2851,13 @@
         <v>175</v>
       </c>
       <c r="D2" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="E2">
         <v>0.98</v>
       </c>
       <c r="F2" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="G2">
         <v>1.03</v>
@@ -2878,7 +2874,7 @@
         <v>201</v>
       </c>
       <c r="F3" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="G3">
         <v>1</v>
@@ -2895,7 +2891,7 @@
         <v>197</v>
       </c>
       <c r="F4" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="G4">
         <v>1.01</v>
@@ -2909,7 +2905,7 @@
         <v>2026</v>
       </c>
       <c r="C5" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="D5" t="s">
         <v>62</v>
@@ -2960,7 +2956,7 @@
     </row>
     <row r="18" spans="10:10">
       <c r="J18" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
     </row>
   </sheetData>
@@ -2989,16 +2985,16 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="C1" t="s">
         <v>160</v>
       </c>
       <c r="D1" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="E1" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -3006,7 +3002,7 @@
         <v>306</v>
       </c>
       <c r="B2" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="C2" t="s">
         <v>174</v>
@@ -3023,7 +3019,7 @@
         <v>14</v>
       </c>
       <c r="B3" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="C3" t="s">
         <v>174</v>
@@ -3061,37 +3057,37 @@
         <v>7</v>
       </c>
       <c r="C1" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="D1" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="E1" t="s">
         <v>164</v>
       </c>
       <c r="F1" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="G1" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="H1" t="s">
         <v>253</v>
       </c>
       <c r="I1" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="J1" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="K1" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="L1" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="M1" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
     </row>
     <row r="2" spans="1:13">
@@ -3102,10 +3098,10 @@
         <v>2025</v>
       </c>
       <c r="C2" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="E2" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -3127,7 +3123,7 @@
         <v>2025</v>
       </c>
       <c r="C4" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="D4" t="s">
         <v>149</v>
@@ -3153,7 +3149,7 @@
         <v>2025</v>
       </c>
       <c r="C5" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="D5" t="s">
         <v>151</v>
@@ -3271,7 +3267,7 @@
     </row>
     <row r="2" spans="1:10">
       <c r="A2" s="5" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="B2" s="5">
         <v>171719833</v>
@@ -3303,7 +3299,7 @@
     </row>
     <row r="3" spans="1:10">
       <c r="A3" s="5" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="B3">
         <v>171770507</v>
@@ -3321,13 +3317,13 @@
         <v>13</v>
       </c>
       <c r="G3" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="H3">
         <v>2026</v>
       </c>
       <c r="I3" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
     </row>
   </sheetData>
@@ -3518,7 +3514,7 @@
         <v>26</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>28</v>
@@ -3538,7 +3534,7 @@
         <v>26</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="I3" s="2" t="s">
         <v>28</v>
@@ -3558,7 +3554,7 @@
         <v>26</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>28</v>
@@ -3578,7 +3574,7 @@
         <v>26</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="I5" s="2" t="s">
         <v>28</v>
@@ -3601,7 +3597,7 @@
         <v>26</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>28</v>
@@ -3621,7 +3617,7 @@
         <v>26</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="I7" s="2" t="s">
         <v>28</v>
@@ -3635,7 +3631,7 @@
         <v>2026</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -3655,7 +3651,7 @@
         <v>26</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="I9" s="2" t="s">
         <v>28</v>
@@ -3675,7 +3671,7 @@
         <v>26</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="I10" s="2" t="s">
         <v>28</v>
@@ -3695,7 +3691,7 @@
         <v>26</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="I11" s="2" t="s">
         <v>28</v>
@@ -3715,7 +3711,7 @@
         <v>26</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="I12" s="2" t="s">
         <v>28</v>
@@ -3738,7 +3734,7 @@
         <v>26</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="I13" s="2" t="s">
         <v>28</v>
@@ -3761,7 +3757,7 @@
         <v>26</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="I14" s="2" t="s">
         <v>28</v>
@@ -3784,7 +3780,7 @@
         <v>26</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="I15" s="2" t="s">
         <v>28</v>
@@ -3804,7 +3800,7 @@
         <v>26</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="I16" s="2" t="s">
         <v>28</v>
@@ -3827,7 +3823,7 @@
         <v>26</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="I17" s="2" t="s">
         <v>28</v>
@@ -3850,7 +3846,7 @@
         <v>26</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="I18" s="2" t="s">
         <v>28</v>
@@ -3873,7 +3869,7 @@
         <v>26</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="I19" s="2" t="s">
         <v>28</v>
@@ -3896,7 +3892,7 @@
         <v>26</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="I20" s="2" t="s">
         <v>28</v>
@@ -3916,7 +3912,7 @@
         <v>26</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="I21" s="2" t="s">
         <v>28</v>
@@ -3936,7 +3932,7 @@
         <v>26</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="I22" s="2" t="s">
         <v>28</v>
@@ -3956,7 +3952,7 @@
         <v>26</v>
       </c>
       <c r="F23" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="I23" s="2" t="s">
         <v>28</v>
@@ -3976,7 +3972,7 @@
         <v>26</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="I24" s="2" t="s">
         <v>28</v>
@@ -3990,13 +3986,13 @@
         <v>141</v>
       </c>
       <c r="C25" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="E25" t="s">
         <v>26</v>
       </c>
       <c r="F25" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="I25" s="2" t="s">
         <v>28</v>
@@ -4010,13 +4006,13 @@
         <v>24</v>
       </c>
       <c r="C26" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>26</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="I26" s="2" t="s">
         <v>28</v>
@@ -4030,13 +4026,13 @@
         <v>322</v>
       </c>
       <c r="C27" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>26</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="I27" s="2" t="s">
         <v>28</v>
@@ -4050,7 +4046,7 @@
         <v>24</v>
       </c>
       <c r="C28" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>26</v>
@@ -4079,7 +4075,7 @@
         <v>26</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -4104,7 +4100,7 @@
         <v>26</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -4595,7 +4591,7 @@
         <v>149</v>
       </c>
       <c r="G19" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
     </row>
     <row r="20" spans="1:14">
@@ -4748,7 +4744,7 @@
         <v>176</v>
       </c>
       <c r="G28" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="J28" t="s">
         <v>228</v>
@@ -4771,7 +4767,7 @@
         <v>176</v>
       </c>
       <c r="G29" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="J29" t="s">
         <v>228</v>
@@ -4794,7 +4790,7 @@
         <v>176</v>
       </c>
       <c r="G30" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="J30" t="s">
         <v>228</v>
@@ -4814,10 +4810,10 @@
         <v>176</v>
       </c>
       <c r="G31" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="M31">
         <v>1280</v>
@@ -4825,7 +4821,7 @@
     </row>
     <row r="58" spans="1:13">
       <c r="G58" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="J58" t="s">
         <v>178</v>
@@ -4833,7 +4829,7 @@
     </row>
     <row r="59" spans="1:13">
       <c r="G59" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
     </row>
     <row r="60" spans="1:13">
@@ -4843,7 +4839,7 @@
     </row>
     <row r="62" spans="1:13">
       <c r="A62" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="B62" t="s">
         <v>172</v>
@@ -4860,7 +4856,7 @@
     </row>
     <row r="63" spans="1:13">
       <c r="A63" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="B63" t="s">
         <v>172</v>
@@ -4872,10 +4868,10 @@
         <v>172</v>
       </c>
       <c r="G63" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="J63" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="K63" t="s">
         <v>62</v>
@@ -6725,6 +6721,12 @@
       <c r="G29" s="10" t="s">
         <v>225</v>
       </c>
+      <c r="H29" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="I29" s="8">
+        <v>640</v>
+      </c>
       <c r="M29" t="s">
         <v>195</v>
       </c>
@@ -8088,13 +8090,13 @@
         <v>323</v>
       </c>
       <c r="J25" t="s">
-        <v>330</v>
+        <v>340</v>
       </c>
       <c r="K25" t="s">
         <v>312</v>
       </c>
       <c r="L25" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
     </row>
     <row r="26" spans="1:12">
@@ -8156,34 +8158,34 @@
         <v>8</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="E1" s="6" t="s">
         <v>236</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="J1" s="6" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="K1" s="6" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="L1" s="6" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="M1" s="6" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
     </row>
     <row r="2" hidden="1" spans="1:13">
@@ -8255,7 +8257,7 @@
         <v>1.1</v>
       </c>
       <c r="J4" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="M4">
         <v>1.9</v>
@@ -8353,34 +8355,34 @@
         <v>8</v>
       </c>
       <c r="D1" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="E1" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="F1" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="G1" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="H1" t="s">
         <v>293</v>
       </c>
       <c r="I1" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="J1" s="9" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="K1" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="L1" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="M1" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
     </row>
     <row r="2" spans="1:13">
@@ -8394,7 +8396,7 @@
         <v>175</v>
       </c>
       <c r="D2" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="E2">
         <v>135</v>
@@ -8409,7 +8411,7 @@
         <v>240</v>
       </c>
       <c r="L2" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="M2">
         <v>10</v>
@@ -8426,7 +8428,7 @@
         <v>175</v>
       </c>
       <c r="D3" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="E3">
         <v>118</v>
@@ -8441,7 +8443,7 @@
         <v>240</v>
       </c>
       <c r="L3" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="M3">
         <v>10</v>
@@ -8458,7 +8460,7 @@
         <v>175</v>
       </c>
       <c r="D4" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="E4">
         <v>96</v>
@@ -8473,7 +8475,7 @@
         <v>240</v>
       </c>
       <c r="L4" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="M4">
         <v>10</v>
@@ -8490,7 +8492,7 @@
         <v>175</v>
       </c>
       <c r="D5" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="E5">
         <v>93</v>
@@ -8505,7 +8507,7 @@
         <v>240</v>
       </c>
       <c r="L5" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="M5">
         <v>10</v>
@@ -8522,7 +8524,7 @@
         <v>175</v>
       </c>
       <c r="D6" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="E6">
         <v>176</v>
@@ -8537,7 +8539,7 @@
         <v>240</v>
       </c>
       <c r="L6" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="M6">
         <v>10</v>
@@ -8569,7 +8571,7 @@
         <v>240</v>
       </c>
       <c r="L7" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="M7">
         <v>10</v>
@@ -8586,7 +8588,7 @@
         <v>175</v>
       </c>
       <c r="D8" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="E8">
         <v>128</v>
@@ -8601,7 +8603,7 @@
         <v>240</v>
       </c>
       <c r="L8" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="M8">
         <v>10</v>
@@ -8618,7 +8620,7 @@
         <v>197</v>
       </c>
       <c r="D9" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="E9">
         <v>128</v>
@@ -8630,19 +8632,19 @@
         <v>63</v>
       </c>
       <c r="H9" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="I9" t="s">
         <v>179</v>
       </c>
       <c r="J9" s="9" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="K9" t="s">
         <v>240</v>
       </c>
       <c r="L9" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="M9">
         <v>2</v>
@@ -8659,7 +8661,7 @@
         <v>199</v>
       </c>
       <c r="D10" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="E10">
         <v>128</v>
@@ -8674,7 +8676,7 @@
         <v>240</v>
       </c>
       <c r="L10" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="M10">
         <v>10</v>

</xml_diff>